<commit_message>
Ajuste na leitura do fgts
</commit_message>
<xml_diff>
--- a/static/planilhas/dados_fgts.xlsx
+++ b/static/planilhas/dados_fgts.xlsx
@@ -441,12 +441,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>62576830 CONDOMINIO EDIFICIO JULIANA</t>
+          <t>62.576.830</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>62.576.830 CONDOMINIO EDIFICIO JULIANA às 21:59:59 (Brasília)</t>
+          <t>CONDOMINIO EDIFICIO JULIANA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -463,12 +463,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>07022952 CONDOMINIO DO EDIFICIO RESIDENCIAL QUINTELA</t>
+          <t>07.022.952</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>07.022.952 CONDOMINIO DO EDIFICIO RESIDENCIAL QUINTELA às 21:59:59 (Brasília)</t>
+          <t>CONDOMINIO DO EDIFICIO RESIDENCIAL QUINTELA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -485,12 +485,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>68760388 CONDOMINIO DO EDIFICIO SABIN</t>
+          <t>68.760.388</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>68.760.388 CONDOMINIO DO EDIFICIO SABIN às 21:59:59 (Brasília)</t>
+          <t>CONDOMINIO DO EDIFICIO SABIN</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">

</xml_diff>